<commit_message>
Add cards-links block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 12
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-campaign-handbook.report.xlsx
+++ b/tools/importer/reports/import-campaign-handbook.report.xlsx
@@ -64,7 +64,7 @@
     <t>campaigns/id-cross.report.json</t>
   </si>
   <si>
-    <t>["hero-campaign","columns-info","cards-features","cards-features"]</t>
+    <t>["hero-campaign","columns-info","cards-features","cards-features","cards-links"]</t>
   </si>
   <si>
     <t>campaigns/id-cross</t>
@@ -73,7 +73,7 @@
     <t>campaign-handbook</t>
   </si>
   <si>
-    <t>2026-10-21T09:39:40.683Z</t>
+    <t>2026-10-21T10:37:09.116Z</t>
   </si>
   <si>
     <t>ID. Cross — Campaign Handbook | Content Shop</t>

</xml_diff>